<commit_message>
feat: adicionar dia 04/10 fechando semana 28 a 04 e recuperacao de 41 lojas em varredura
</commit_message>
<xml_diff>
--- a/dados_all_stores/KEYS Service Exceptions - All Stores (Stores) (2026-10-02).xlsx
+++ b/dados_all_stores/KEYS Service Exceptions - All Stores (Stores) (2026-10-02).xlsx
@@ -935,43 +935,43 @@
     <t>214</t>
   </si>
   <si>
-    <t>40</t>
-  </si>
-  <si>
-    <t>R$ 9.681,64</t>
+    <t>37</t>
+  </si>
+  <si>
+    <t>R$ 9.689,76</t>
   </si>
   <si>
     <t>101.4</t>
   </si>
   <si>
-    <t>70.6</t>
-  </si>
-  <si>
-    <t>6.40</t>
-  </si>
-  <si>
-    <t>21.7</t>
-  </si>
-  <si>
-    <t>8.6</t>
-  </si>
-  <si>
-    <t>5.8</t>
-  </si>
-  <si>
-    <t>30.5%</t>
-  </si>
-  <si>
-    <t>18.3%</t>
-  </si>
-  <si>
-    <t>1.3%</t>
+    <t>70.7</t>
+  </si>
+  <si>
+    <t>6.49</t>
+  </si>
+  <si>
+    <t>21.9</t>
+  </si>
+  <si>
+    <t>8.7</t>
+  </si>
+  <si>
+    <t>5.9</t>
+  </si>
+  <si>
+    <t>30.1%</t>
+  </si>
+  <si>
+    <t>18.6%</t>
+  </si>
+  <si>
+    <t>1.4%</t>
   </si>
   <si>
     <t>0.2%</t>
   </si>
   <si>
-    <t>3.6%</t>
+    <t>3.5%</t>
   </si>
   <si>
     <t>1.1%</t>
@@ -980,46 +980,46 @@
     <t>6.2%</t>
   </si>
   <si>
-    <t>2.2%</t>
-  </si>
-  <si>
-    <t>7.5%</t>
-  </si>
-  <si>
-    <t>2726.0</t>
-  </si>
-  <si>
-    <t>2206.0</t>
-  </si>
-  <si>
-    <t>163.0</t>
-  </si>
-  <si>
-    <t>23.0</t>
-  </si>
-  <si>
-    <t>430.0</t>
-  </si>
-  <si>
-    <t>134.0</t>
-  </si>
-  <si>
-    <t>22.0</t>
-  </si>
-  <si>
-    <t>749.0</t>
-  </si>
-  <si>
-    <t>271.0</t>
-  </si>
-  <si>
-    <t>908.0</t>
-  </si>
-  <si>
-    <t>0.4%</t>
-  </si>
-  <si>
-    <t>49.0</t>
+    <t>2.3%</t>
+  </si>
+  <si>
+    <t>7.7%</t>
+  </si>
+  <si>
+    <t>2835.0</t>
+  </si>
+  <si>
+    <t>2306.0</t>
+  </si>
+  <si>
+    <t>169.0</t>
+  </si>
+  <si>
+    <t>26.0</t>
+  </si>
+  <si>
+    <t>438.0</t>
+  </si>
+  <si>
+    <t>137.0</t>
+  </si>
+  <si>
+    <t>24.0</t>
+  </si>
+  <si>
+    <t>762.0</t>
+  </si>
+  <si>
+    <t>289.0</t>
+  </si>
+  <si>
+    <t>955.0</t>
+  </si>
+  <si>
+    <t>0.5%</t>
+  </si>
+  <si>
+    <t>61.0</t>
   </si>
   <si>
     <t>1</t>
@@ -3239,7 +3239,7 @@
         <v>19515</v>
       </c>
       <c r="B13" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c t="s" r="C13" s="4">
         <v>51</v>
@@ -3269,35 +3269,93 @@
         <v>58</v>
       </c>
       <c r="L13" s="4"/>
-      <c r="M13" s="5"/>
-      <c r="N13" s="6"/>
-      <c r="O13" s="6"/>
-      <c r="P13" s="7"/>
-      <c r="Q13" s="8"/>
-      <c r="R13" s="8"/>
-      <c r="S13" s="8"/>
-      <c r="T13" s="9"/>
-      <c r="U13" s="9"/>
-      <c r="V13" s="9"/>
-      <c r="W13" s="9"/>
-      <c r="X13" s="9"/>
-      <c r="Y13" s="9"/>
-      <c r="Z13" s="9"/>
-      <c r="AA13" s="9"/>
-      <c r="AB13" s="9"/>
-      <c r="AC13" s="9"/>
-      <c r="AD13" s="6"/>
-      <c r="AE13" s="6"/>
-      <c r="AF13" s="6"/>
-      <c r="AG13" s="6"/>
-      <c r="AH13" s="6"/>
-      <c r="AI13" s="6"/>
-      <c r="AJ13" s="6"/>
-      <c r="AK13" s="6"/>
-      <c r="AL13" s="6"/>
-      <c r="AM13" s="6"/>
-      <c r="AN13" s="9"/>
-      <c r="AO13" s="6"/>
+      <c r="M13" s="5">
+        <v>15512</v>
+      </c>
+      <c r="N13" s="6">
+        <v>162</v>
+      </c>
+      <c r="O13" s="6">
+        <v>130</v>
+      </c>
+      <c r="P13" s="7">
+        <v>14.067272727272726</v>
+      </c>
+      <c r="Q13" s="8">
+        <v>29.772307692307692</v>
+      </c>
+      <c r="R13" s="8">
+        <v>7.4516669230769228</v>
+      </c>
+      <c r="S13" s="8">
+        <v>7</v>
+      </c>
+      <c r="T13" s="9">
+        <v>0.13846153846153847</v>
+      </c>
+      <c r="U13" s="9">
+        <v>0.23846153846153847</v>
+      </c>
+      <c r="V13" s="9">
+        <v>0.015384615384615385</v>
+      </c>
+      <c r="W13" s="9">
+        <v>0</v>
+      </c>
+      <c r="X13" s="9">
+        <v>0.023076923076923078</v>
+      </c>
+      <c r="Y13" s="9">
+        <v>0</v>
+      </c>
+      <c r="Z13" s="9">
+        <v>0</v>
+      </c>
+      <c r="AA13" s="9">
+        <v>0</v>
+      </c>
+      <c r="AB13" s="9">
+        <v>0.038461538461538464</v>
+      </c>
+      <c r="AC13" s="9">
+        <v>0.076923076923076927</v>
+      </c>
+      <c r="AD13" s="6">
+        <v>32</v>
+      </c>
+      <c r="AE13" s="6">
+        <v>31</v>
+      </c>
+      <c r="AF13" s="6">
+        <v>2</v>
+      </c>
+      <c r="AG13" s="6">
+        <v>0</v>
+      </c>
+      <c r="AH13" s="6">
+        <v>3</v>
+      </c>
+      <c r="AI13" s="6">
+        <v>0</v>
+      </c>
+      <c r="AJ13" s="6">
+        <v>0</v>
+      </c>
+      <c r="AK13" s="6">
+        <v>0</v>
+      </c>
+      <c r="AL13" s="6">
+        <v>5</v>
+      </c>
+      <c r="AM13" s="6">
+        <v>10</v>
+      </c>
+      <c r="AN13" s="9">
+        <v>0.092307692307692313</v>
+      </c>
+      <c r="AO13" s="6">
+        <v>12</v>
+      </c>
       <c t="s" r="AP13" s="4">
         <v>58</v>
       </c>
@@ -10478,7 +10536,9 @@
       <c r="N62" s="6">
         <v>86</v>
       </c>
-      <c r="O62" s="6"/>
+      <c r="O62" s="6">
+        <v>54</v>
+      </c>
       <c r="P62" s="7">
         <v>3.1877390804597701</v>
       </c>
@@ -10488,31 +10548,75 @@
       <c r="R62" s="8">
         <v>7.0955134615384612</v>
       </c>
-      <c r="S62" s="8"/>
+      <c r="S62" s="8">
+        <v>7</v>
+      </c>
       <c r="T62" s="9">
         <v>0.40740740740740738</v>
       </c>
-      <c r="U62" s="9"/>
-      <c r="V62" s="9"/>
-      <c r="W62" s="9"/>
-      <c r="X62" s="9"/>
-      <c r="Y62" s="9"/>
-      <c r="Z62" s="9"/>
-      <c r="AA62" s="9"/>
-      <c r="AB62" s="9"/>
-      <c r="AC62" s="9"/>
-      <c r="AD62" s="6"/>
-      <c r="AE62" s="6"/>
-      <c r="AF62" s="6"/>
-      <c r="AG62" s="6"/>
-      <c r="AH62" s="6"/>
-      <c r="AI62" s="6"/>
-      <c r="AJ62" s="6"/>
-      <c r="AK62" s="6"/>
-      <c r="AL62" s="6"/>
-      <c r="AM62" s="6"/>
-      <c r="AN62" s="9"/>
-      <c r="AO62" s="6"/>
+      <c r="U62" s="9">
+        <v>0.14814814814814814</v>
+      </c>
+      <c r="V62" s="9">
+        <v>0</v>
+      </c>
+      <c r="W62" s="9">
+        <v>0</v>
+      </c>
+      <c r="X62" s="9">
+        <v>0.092592592592592587</v>
+      </c>
+      <c r="Y62" s="9">
+        <v>0.018518518518518517</v>
+      </c>
+      <c r="Z62" s="9">
+        <v>0.037037037037037035</v>
+      </c>
+      <c r="AA62" s="9">
+        <v>0.037037037037037035</v>
+      </c>
+      <c r="AB62" s="9">
+        <v>0.037037037037037035</v>
+      </c>
+      <c r="AC62" s="9">
+        <v>0</v>
+      </c>
+      <c r="AD62" s="6">
+        <v>12</v>
+      </c>
+      <c r="AE62" s="6">
+        <v>8</v>
+      </c>
+      <c r="AF62" s="6">
+        <v>0</v>
+      </c>
+      <c r="AG62" s="6">
+        <v>0</v>
+      </c>
+      <c r="AH62" s="6">
+        <v>5</v>
+      </c>
+      <c r="AI62" s="6">
+        <v>1</v>
+      </c>
+      <c r="AJ62" s="6">
+        <v>2</v>
+      </c>
+      <c r="AK62" s="6">
+        <v>2</v>
+      </c>
+      <c r="AL62" s="6">
+        <v>2</v>
+      </c>
+      <c r="AM62" s="6">
+        <v>0</v>
+      </c>
+      <c r="AN62" s="9">
+        <v>0</v>
+      </c>
+      <c r="AO62" s="6">
+        <v>0</v>
+      </c>
       <c t="s" r="AP62" s="4">
         <v>58</v>
       </c>
@@ -14418,7 +14522,7 @@
         <v>19694</v>
       </c>
       <c r="B90" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c t="s" r="C90" s="4">
         <v>51</v>
@@ -14448,35 +14552,93 @@
         <v>58</v>
       </c>
       <c r="L90" s="4"/>
-      <c r="M90" s="5"/>
-      <c r="N90" s="6"/>
-      <c r="O90" s="6"/>
-      <c r="P90" s="7"/>
-      <c r="Q90" s="8"/>
-      <c r="R90" s="8"/>
-      <c r="S90" s="8"/>
-      <c r="T90" s="9"/>
-      <c r="U90" s="9"/>
-      <c r="V90" s="9"/>
-      <c r="W90" s="9"/>
-      <c r="X90" s="9"/>
-      <c r="Y90" s="9"/>
-      <c r="Z90" s="9"/>
-      <c r="AA90" s="9"/>
-      <c r="AB90" s="9"/>
-      <c r="AC90" s="9"/>
-      <c r="AD90" s="6"/>
-      <c r="AE90" s="6"/>
-      <c r="AF90" s="6"/>
-      <c r="AG90" s="6"/>
-      <c r="AH90" s="6"/>
-      <c r="AI90" s="6"/>
-      <c r="AJ90" s="6"/>
-      <c r="AK90" s="6"/>
-      <c r="AL90" s="6"/>
-      <c r="AM90" s="6"/>
-      <c r="AN90" s="9"/>
-      <c r="AO90" s="6"/>
+      <c r="M90" s="5">
+        <v>8103.5299999999997</v>
+      </c>
+      <c r="N90" s="6">
+        <v>79</v>
+      </c>
+      <c r="O90" s="6">
+        <v>62</v>
+      </c>
+      <c r="P90" s="7">
+        <v>14.025406097560976</v>
+      </c>
+      <c r="Q90" s="8">
+        <v>42.885483870967747</v>
+      </c>
+      <c r="R90" s="8">
+        <v>21.194624193548389</v>
+      </c>
+      <c r="S90" s="8">
+        <v>7</v>
+      </c>
+      <c r="T90" s="9">
+        <v>0.032258064516129031</v>
+      </c>
+      <c r="U90" s="9">
+        <v>0.66129032258064513</v>
+      </c>
+      <c r="V90" s="9">
+        <v>0.064516129032258063</v>
+      </c>
+      <c r="W90" s="9">
+        <v>0</v>
+      </c>
+      <c r="X90" s="9">
+        <v>0</v>
+      </c>
+      <c r="Y90" s="9">
+        <v>0</v>
+      </c>
+      <c r="Z90" s="9">
+        <v>0</v>
+      </c>
+      <c r="AA90" s="9">
+        <v>0</v>
+      </c>
+      <c r="AB90" s="9">
+        <v>0.17741935483870969</v>
+      </c>
+      <c r="AC90" s="9">
+        <v>0.45161290322580644</v>
+      </c>
+      <c r="AD90" s="6">
+        <v>43</v>
+      </c>
+      <c r="AE90" s="6">
+        <v>41</v>
+      </c>
+      <c r="AF90" s="6">
+        <v>4</v>
+      </c>
+      <c r="AG90" s="6">
+        <v>0</v>
+      </c>
+      <c r="AH90" s="6">
+        <v>0</v>
+      </c>
+      <c r="AI90" s="6">
+        <v>0</v>
+      </c>
+      <c r="AJ90" s="6">
+        <v>0</v>
+      </c>
+      <c r="AK90" s="6">
+        <v>0</v>
+      </c>
+      <c r="AL90" s="6">
+        <v>11</v>
+      </c>
+      <c r="AM90" s="6">
+        <v>28</v>
+      </c>
+      <c r="AN90" s="9">
+        <v>0</v>
+      </c>
+      <c r="AO90" s="6">
+        <v>0</v>
+      </c>
       <c t="s" r="AP90" s="4">
         <v>58</v>
       </c>
@@ -16176,7 +16338,7 @@
         <v>19719</v>
       </c>
       <c r="B102" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c t="s" r="C102" s="4">
         <v>51</v>
@@ -16206,35 +16368,93 @@
         <v>58</v>
       </c>
       <c r="L102" s="4"/>
-      <c r="M102" s="5"/>
-      <c r="N102" s="6"/>
-      <c r="O102" s="6"/>
-      <c r="P102" s="7"/>
-      <c r="Q102" s="8"/>
-      <c r="R102" s="8"/>
-      <c r="S102" s="8"/>
-      <c r="T102" s="9"/>
-      <c r="U102" s="9"/>
-      <c r="V102" s="9"/>
-      <c r="W102" s="9"/>
-      <c r="X102" s="9"/>
-      <c r="Y102" s="9"/>
-      <c r="Z102" s="9"/>
-      <c r="AA102" s="9"/>
-      <c r="AB102" s="9"/>
-      <c r="AC102" s="9"/>
-      <c r="AD102" s="6"/>
-      <c r="AE102" s="6"/>
-      <c r="AF102" s="6"/>
-      <c r="AG102" s="6"/>
-      <c r="AH102" s="6"/>
-      <c r="AI102" s="6"/>
-      <c r="AJ102" s="6"/>
-      <c r="AK102" s="6"/>
-      <c r="AL102" s="6"/>
-      <c r="AM102" s="6"/>
-      <c r="AN102" s="9"/>
-      <c r="AO102" s="6"/>
+      <c r="M102" s="5">
+        <v>6858.21</v>
+      </c>
+      <c r="N102" s="6">
+        <v>77</v>
+      </c>
+      <c r="O102" s="6">
+        <v>55</v>
+      </c>
+      <c r="P102" s="7">
+        <v>6.7989716049382709</v>
+      </c>
+      <c r="Q102" s="8">
+        <v>18.919090909090908</v>
+      </c>
+      <c r="R102" s="8">
+        <v>6.9260416666666664</v>
+      </c>
+      <c r="S102" s="8">
+        <v>7</v>
+      </c>
+      <c r="T102" s="9">
+        <v>0.29090909090909089</v>
+      </c>
+      <c r="U102" s="9">
+        <v>0.36363636363636365</v>
+      </c>
+      <c r="V102" s="9">
+        <v>0</v>
+      </c>
+      <c r="W102" s="9">
+        <v>0.054545454544999997</v>
+      </c>
+      <c r="X102" s="9">
+        <v>0</v>
+      </c>
+      <c r="Y102" s="9">
+        <v>0.036363636363636362</v>
+      </c>
+      <c r="Z102" s="9">
+        <v>0</v>
+      </c>
+      <c r="AA102" s="9">
+        <v>0.20000000000000001</v>
+      </c>
+      <c r="AB102" s="9">
+        <v>0</v>
+      </c>
+      <c r="AC102" s="9">
+        <v>0.16363636363636364</v>
+      </c>
+      <c r="AD102" s="6">
+        <v>22</v>
+      </c>
+      <c r="AE102" s="6">
+        <v>20</v>
+      </c>
+      <c r="AF102" s="6">
+        <v>0</v>
+      </c>
+      <c r="AG102" s="6">
+        <v>3</v>
+      </c>
+      <c r="AH102" s="6">
+        <v>0</v>
+      </c>
+      <c r="AI102" s="6">
+        <v>2</v>
+      </c>
+      <c r="AJ102" s="6">
+        <v>0</v>
+      </c>
+      <c r="AK102" s="6">
+        <v>11</v>
+      </c>
+      <c r="AL102" s="6">
+        <v>0</v>
+      </c>
+      <c r="AM102" s="6">
+        <v>9</v>
+      </c>
+      <c r="AN102" s="9">
+        <v>0</v>
+      </c>
+      <c r="AO102" s="6">
+        <v>0</v>
+      </c>
       <c t="s" r="AP102" s="4">
         <v>58</v>
       </c>

</xml_diff>

<commit_message>
feat: varredura e atualizacao ate 09/10 com 50 lojas e 2800 pedidos recuperados e novos dias 08 e 09/10
</commit_message>
<xml_diff>
--- a/dados_all_stores/KEYS Service Exceptions - All Stores (Stores) (2026-10-02).xlsx
+++ b/dados_all_stores/KEYS Service Exceptions - All Stores (Stores) (2026-10-02).xlsx
@@ -935,22 +935,22 @@
     <t>214</t>
   </si>
   <si>
-    <t>32</t>
-  </si>
-  <si>
-    <t>R$ 9.764,04</t>
-  </si>
-  <si>
-    <t>101.5</t>
-  </si>
-  <si>
-    <t>71.2</t>
-  </si>
-  <si>
-    <t>6.51</t>
-  </si>
-  <si>
-    <t>22.0</t>
+    <t>30</t>
+  </si>
+  <si>
+    <t>R$ 9.778,97</t>
+  </si>
+  <si>
+    <t>101.7</t>
+  </si>
+  <si>
+    <t>71.5</t>
+  </si>
+  <si>
+    <t>6.54</t>
+  </si>
+  <si>
+    <t>22.1</t>
   </si>
   <si>
     <t>8.8</t>
@@ -959,10 +959,10 @@
     <t>6.1</t>
   </si>
   <si>
-    <t>29.7%</t>
-  </si>
-  <si>
-    <t>18.3%</t>
+    <t>29.5%</t>
+  </si>
+  <si>
+    <t>18.1%</t>
   </si>
   <si>
     <t>1.3%</t>
@@ -977,28 +977,28 @@
     <t>1.1%</t>
   </si>
   <si>
-    <t>6.0%</t>
+    <t>5.9%</t>
   </si>
   <si>
     <t>2.3%</t>
   </si>
   <si>
-    <t>7.6%</t>
-  </si>
-  <si>
-    <t>2880.0</t>
-  </si>
-  <si>
-    <t>2347.0</t>
-  </si>
-  <si>
-    <t>170.0</t>
+    <t>7.5%</t>
+  </si>
+  <si>
+    <t>2891.0</t>
+  </si>
+  <si>
+    <t>2358.0</t>
+  </si>
+  <si>
+    <t>175.0</t>
   </si>
   <si>
     <t>26.0</t>
   </si>
   <si>
-    <t>448.0</t>
+    <t>449.0</t>
   </si>
   <si>
     <t>137.0</t>
@@ -1007,13 +1007,13 @@
     <t>25.0</t>
   </si>
   <si>
-    <t>769.0</t>
+    <t>772.0</t>
   </si>
   <si>
     <t>297.0</t>
   </si>
   <si>
-    <t>973.0</t>
+    <t>975.0</t>
   </si>
   <si>
     <t>0.5%</t>
@@ -6782,7 +6782,7 @@
         <v>19562</v>
       </c>
       <c r="B36" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c t="s" r="C36" s="4">
         <v>51</v>
@@ -6812,35 +6812,93 @@
         <v>58</v>
       </c>
       <c r="L36" s="4"/>
-      <c r="M36" s="5"/>
-      <c r="N36" s="6"/>
-      <c r="O36" s="6"/>
-      <c r="P36" s="7"/>
-      <c r="Q36" s="8"/>
-      <c r="R36" s="8"/>
-      <c r="S36" s="8"/>
-      <c r="T36" s="9"/>
-      <c r="U36" s="9"/>
-      <c r="V36" s="9"/>
-      <c r="W36" s="9"/>
-      <c r="X36" s="9"/>
-      <c r="Y36" s="9"/>
-      <c r="Z36" s="9"/>
-      <c r="AA36" s="9"/>
-      <c r="AB36" s="9"/>
-      <c r="AC36" s="9"/>
-      <c r="AD36" s="6"/>
-      <c r="AE36" s="6"/>
-      <c r="AF36" s="6"/>
-      <c r="AG36" s="6"/>
-      <c r="AH36" s="6"/>
-      <c r="AI36" s="6"/>
-      <c r="AJ36" s="6"/>
-      <c r="AK36" s="6"/>
-      <c r="AL36" s="6"/>
-      <c r="AM36" s="6"/>
-      <c r="AN36" s="9"/>
-      <c r="AO36" s="6"/>
+      <c r="M36" s="5">
+        <v>10427.73</v>
+      </c>
+      <c r="N36" s="6">
+        <v>129</v>
+      </c>
+      <c r="O36" s="6">
+        <v>108</v>
+      </c>
+      <c r="P36" s="7">
+        <v>10.762132352941178</v>
+      </c>
+      <c r="Q36" s="8">
+        <v>38.06898148148148</v>
+      </c>
+      <c r="R36" s="8">
+        <v>20.381775700934579</v>
+      </c>
+      <c r="S36" s="8">
+        <v>7</v>
+      </c>
+      <c r="T36" s="9">
+        <v>0.083333333333333329</v>
+      </c>
+      <c r="U36" s="9">
+        <v>0.027777777777777776</v>
+      </c>
+      <c r="V36" s="9">
+        <v>0.0092592592592592587</v>
+      </c>
+      <c r="W36" s="9">
+        <v>0</v>
+      </c>
+      <c r="X36" s="9">
+        <v>0.0092592592592592587</v>
+      </c>
+      <c r="Y36" s="9">
+        <v>0</v>
+      </c>
+      <c r="Z36" s="9">
+        <v>0</v>
+      </c>
+      <c r="AA36" s="9">
+        <v>0.0092592592592592587</v>
+      </c>
+      <c r="AB36" s="9">
+        <v>0</v>
+      </c>
+      <c r="AC36" s="9">
+        <v>0</v>
+      </c>
+      <c r="AD36" s="6">
+        <v>3</v>
+      </c>
+      <c r="AE36" s="6">
+        <v>3</v>
+      </c>
+      <c r="AF36" s="6">
+        <v>1</v>
+      </c>
+      <c r="AG36" s="6">
+        <v>0</v>
+      </c>
+      <c r="AH36" s="6">
+        <v>1</v>
+      </c>
+      <c r="AI36" s="6">
+        <v>0</v>
+      </c>
+      <c r="AJ36" s="6">
+        <v>0</v>
+      </c>
+      <c r="AK36" s="6">
+        <v>1</v>
+      </c>
+      <c r="AL36" s="6">
+        <v>0</v>
+      </c>
+      <c r="AM36" s="6">
+        <v>0</v>
+      </c>
+      <c r="AN36" s="9">
+        <v>0</v>
+      </c>
+      <c r="AO36" s="6">
+        <v>0</v>
+      </c>
       <c t="s" r="AP36" s="4">
         <v>58</v>
       </c>
@@ -7664,7 +7722,7 @@
         <v>19579</v>
       </c>
       <c r="B42" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c t="s" r="C42" s="4">
         <v>51</v>
@@ -7694,35 +7752,93 @@
         <v>58</v>
       </c>
       <c r="L42" s="4"/>
-      <c r="M42" s="5"/>
-      <c r="N42" s="6"/>
-      <c r="O42" s="6"/>
-      <c r="P42" s="7"/>
-      <c r="Q42" s="8"/>
-      <c r="R42" s="8"/>
-      <c r="S42" s="8"/>
-      <c r="T42" s="9"/>
-      <c r="U42" s="9"/>
-      <c r="V42" s="9"/>
-      <c r="W42" s="9"/>
-      <c r="X42" s="9"/>
-      <c r="Y42" s="9"/>
-      <c r="Z42" s="9"/>
-      <c r="AA42" s="9"/>
-      <c r="AB42" s="9"/>
-      <c r="AC42" s="9"/>
-      <c r="AD42" s="6"/>
-      <c r="AE42" s="6"/>
-      <c r="AF42" s="6"/>
-      <c r="AG42" s="6"/>
-      <c r="AH42" s="6"/>
-      <c r="AI42" s="6"/>
-      <c r="AJ42" s="6"/>
-      <c r="AK42" s="6"/>
-      <c r="AL42" s="6"/>
-      <c r="AM42" s="6"/>
-      <c r="AN42" s="9"/>
-      <c r="AO42" s="6"/>
+      <c r="M42" s="5">
+        <v>11818.24</v>
+      </c>
+      <c r="N42" s="6">
+        <v>122</v>
+      </c>
+      <c r="O42" s="6">
+        <v>88</v>
+      </c>
+      <c r="P42" s="7">
+        <v>6.0912353448275862</v>
+      </c>
+      <c r="Q42" s="8">
+        <v>21.254980459770113</v>
+      </c>
+      <c r="R42" s="8">
+        <v>8.1312264367816098</v>
+      </c>
+      <c r="S42" s="8">
+        <v>7</v>
+      </c>
+      <c r="T42" s="9">
+        <v>0.25287356321839083</v>
+      </c>
+      <c r="U42" s="9">
+        <v>0.090909090909090912</v>
+      </c>
+      <c r="V42" s="9">
+        <v>0.045454545454545456</v>
+      </c>
+      <c r="W42" s="9">
+        <v>0</v>
+      </c>
+      <c r="X42" s="9">
+        <v>0</v>
+      </c>
+      <c r="Y42" s="9">
+        <v>0</v>
+      </c>
+      <c r="Z42" s="9">
+        <v>0</v>
+      </c>
+      <c r="AA42" s="9">
+        <v>0.022727272727272728</v>
+      </c>
+      <c r="AB42" s="9">
+        <v>0</v>
+      </c>
+      <c r="AC42" s="9">
+        <v>0.022727272727272728</v>
+      </c>
+      <c r="AD42" s="6">
+        <v>8</v>
+      </c>
+      <c r="AE42" s="6">
+        <v>8</v>
+      </c>
+      <c r="AF42" s="6">
+        <v>4</v>
+      </c>
+      <c r="AG42" s="6">
+        <v>0</v>
+      </c>
+      <c r="AH42" s="6">
+        <v>0</v>
+      </c>
+      <c r="AI42" s="6">
+        <v>0</v>
+      </c>
+      <c r="AJ42" s="6">
+        <v>0</v>
+      </c>
+      <c r="AK42" s="6">
+        <v>2</v>
+      </c>
+      <c r="AL42" s="6">
+        <v>0</v>
+      </c>
+      <c r="AM42" s="6">
+        <v>2</v>
+      </c>
+      <c r="AN42" s="9">
+        <v>0</v>
+      </c>
+      <c r="AO42" s="6">
+        <v>0</v>
+      </c>
       <c t="s" r="AP42" s="4">
         <v>58</v>
       </c>

</xml_diff>